<commit_message>
Map 2025 BoA checking inflows onto Consultant, LTR rent, and exclusions.
GCM BOM payments of $21,500 tie the 1099-NEC onto EPGC Consultant; reimbursements, Bear Creek gifts, and UTMA wires stay off income. Joint-account Zelle from Delach, Ava, and Joan is booked on 216 Oak Park rental income, with open questions on the ASK tab.

Co-authored-by: ColeyFineArts <ColeyFineArts@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/.cursor/scratch/tax_turbo_parts/ASK.xlsx
+++ b/.cursor/scratch/tax_turbo_parts/ASK.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B45"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -662,278 +662,545 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>BoA checking folders = 9922 + 0203</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>JSC Adv Plus 4830 6191 9922 (Jake) and joint Adv Plus 4830 7359 0203 (Megan+Jacob). 12 statements each for 2025. Monarch credits on those two accounts match the statement deposit sections sampled.</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>GCM board fee → Consultant</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Gates Capital BOM PAYMEN $21500.00: 2/12 $4,100 + 4/18 $9,200 + 9/13 $4,100 + 11/13 $4,100. Equals Form 1099-NEC $21,500. Booked EPGC Consultant (cash-basis month) and GCM tab. Income tab GCM actual was already $21,500.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>GCM reimbursements EXCLUDED</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>JAKE C / SEFOF on 9922 $3033.83 (board meeting $1,150.99; 5/22 $609.02 unlabeled; 11/05 $1,273.82). Plus Checking 8507 SEFOF $2180.86 (Wharton / annual conference / education committee) — that account is not in the two folders. Total reimbursement $5214.69 kept off Consultant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>LTR rent → 216 Oak Park STR / RENTAL INCOME</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>JOHN T DELACH 8×$1,450 ($11600.00) + Joan Friedberger 2×$1,950 ($3900.00) on joint 0203. Ava L Hernandez 8×$500 ($4000.00) same rent memo / $1,950 combined — included yellow (ASK). TY2025 cash total $19500.00. Oct–Nov 2025: no rent on 0203.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Bear Creek not income</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Four wires $9,500 on Jake 9922 (1/9, 4/10, 7/10, 10/9) = $38000.00. Annual gift — excluded from Consultant / rental / Income tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>UTMA not income</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Emma CMA 2T48 + sibling CMA 4729: Thomas wires $5,000 each Nov/Dec = $10000.00 (not ~$10k each). Treasury-note maturities $10,000 each 12/31 are principal, not gifts. Excluded from income.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24"/>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>STILL OPEN</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>What to confirm</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>REMIND JACOB — ComEd with Megan</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>ComEd is not on these cards. Monarch Adv Plus shows ACH: Jacob Coley $829.15 → Unit 2 ELECTRIC; Megan Gerrard $1,565.26 → Unit 1 ELECTRIC (yellow). User: must have been paid directly or with a check. Double-check with Megan: meters, whether Jake checking ACH is the full picture, and any extra check/direct payments.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Joint 0203 statements show ComEd ACH (e.g. 1/21 Jacob $59.04 + Megan $132.94). ComEd is not on these cards. Monarch Adv Plus shows ACH: Jacob Coley $829.15 → Unit 2 ELECTRIC; Megan Gerrard $1,565.26 → Unit 1 ELECTRIC (yellow). User: must have been paid directly or with a check. Double-check with Megan: meters, whether Jake checking ACH is the full picture, and any extra check/direct payments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>Soldier Field East Parking $57</t>
         </is>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>Coinbase 2025-11-01 same day as Field Museum. Not confirmed — HOLD.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Extra Space $360</t>
         </is>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Prime 2025-12-10. Not part of the HD/Lowe’s/IKEA split — HOLD (storage vs moving vs personal).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>State Farm declarations / Sep–Dec</t>
         </is>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Home vs auto $ is a Feb-charge proxy ($157.53 home / $145.25 auto) until declarations pages. None on Prime Sep–Dec 2025 (524 sold 12/18 — those months may be another account). 2023–24 Excel booked all homeowners on U1; this packet 50/50’s the home share. No 2025 Travelers found on Prime/Sapphire/BoA/Monarch.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Inventory object IDs</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Frame Up $536.41 + LAMA $6,821.06 + Hindman $282.24 + $403.51 parked off Cost total until objects named (avoid Mercury double count).</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>827 N Grove the house — HD 1/3 vs locked CapEx</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>HD/Lowe’s/IKEA 1/3 $604.12 is pre-close materials for 827 N Grove the house (Q5 split), not Grove Collaborative. Do NOT fold into locked TY2025 CapEx $53,660 until CPA says so.</t>
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Ava L Hernandez $500/mo rent</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Eight Zelle credits on joint 0203, same days as Delach, memo “rent”. Delach $1,450 + Ava $500 = $1,950, which is Joan’s later rent. Is Ava Delach’s roommate/co-tenant at 216 Oak Park? I booked her on STR / RENTAL INCOME (yellow) so the $1,950 unit rent is complete. Say if she should be excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Oak Park vacant Oct–Nov 2025?</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>No Delach / Ava / Joan rent on 0203 in October or November. Last Delach/Ava is 8/29 “September Rent”. Joan starts 12/1. Confirm those two months were vacant (and held for rent) for Sch E. Jan 2025 occupancy cash hit 12/31/2024 ($1,450+$500) — left out of TY2025 cash. Correct?</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Joan Friedberger Dec cash</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>12/1 $1,950 memo “rent” and 12/31 $1,950 memo “January rent” both in TY2025 cash. Is 12/1 December occupancy and 12/31 January 2026 prepaid? Also: Checking 8507 Zelle OUT $675 to Joan on 12/1 — deposit return / repair? Not on these two BoA folders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>GCM on EPGC Consultant vs personal 1099</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>You said board fee → consultant line, so I put BOM $21,500 on EPGC LLC Consultant. Historically GCM lived on its own tab + Income “GCM Boards”, and EPGC Consultant was empty. 1099-NEC is in Jacob’s name from Gates Capital. Confirm: EPGC LLC (this booking) vs personal Sch C / GCM tab only (then I will zero EPGC Consultant so LLC P&amp;L is not mixed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>May 22 Gates $609.02</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Statement says GATES CAPITAL MA DES:JAKE C $609.02 — no PMT INFO. Same DES as reimbursements, not BOM PAYMEN. I excluded it from Consultant. Confirm it is reimbursement (or board fee if you say so).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Bear Creek $38,000 vs kids’ UTMA ~$10k each</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Bear Creek to Jake 9922 is $9,500×4 = $38,000 (not ~$10k). Thomas wires into the two CMA-Edge UTMAs are $5,000 each in late Nov. Are Bear Creek gifts to you (parents), and Thomas the kids’ UTMA? Is more UTMA cash coming that never hit these checkings (e.g. directly at Merrill)? 2/25 $36,000 9922→National Financial was reversed 2/27.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Freeman’s / CIBC $11,000 wire 12/24 on joint 0203</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>ORIG:FREEMAN'S LLC via CIBC Bank USA; PMT DET Sale 6428 Contract 303468. Not W-2 payroll (those are DIR DEP on 9922). Art sale? Consignment? Other? HOLD off income until you say.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Checking 8507 (NOW) 2025 statements?</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>Third checking in Monarch — Airbnb/VRBO STR, Megan Zelle, and the three GCM SEFOF reimbursements. Not in the two folders you just added. Upload 2025 statements if you want that account reconciled the same way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Applied / split totals</t>
         </is>
       </c>
-      <c r="B27" s="7" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="B41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
         <is>
           <t>EPGC Travel (Park Chicago $100 + Field Museum $53)</t>
         </is>
       </c>
-      <c r="B28" s="9" t="n">
+      <c r="B42" s="9" t="n">
         <v>153</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>March HD 100% 524 repairs</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="n">
-        <v>1358.65</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Remaining HD/Lowe’s/IKEA (split pool)</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="n">
-        <v>1812.46</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>524 repairs from remaining 1/3 (then 50/50 U1/U2)</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="n">
-        <v>604.1799999999999</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>Unit 2 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="n">
-        <v>981.4400000000001</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>Unit 1 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="n">
-        <v>981.39</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="inlineStr">
-        <is>
-          <t>Personal 1/3 (excluded from P&amp;L)</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="n">
-        <v>604.16</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>827 N Grove the house 1/3 HD/Lowe’s/IKEA (not Grove Collaborative; not locked $53,660)</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="n">
-        <v>604.12</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>524 Unit 2 SUPPLIES (Grove Collaborative)</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="n">
-        <v>791.21</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
-        <is>
-          <t>Unit 2 ELECTRIC ComEd Jacob (YELLOW — ask Megan)</t>
-        </is>
-      </c>
-      <c r="B37" s="13" t="n">
-        <v>829.15</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
-        <is>
-          <t>Unit 1 ELECTRIC ComEd Megan (YELLOW — ask Megan)</t>
-        </is>
-      </c>
-      <c r="B38" s="13" t="n">
-        <v>1565.26</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>524 INSURANCE home share (Unit 2 50%, yellow proxy)</t>
-        </is>
-      </c>
-      <c r="B39" s="15" t="n">
-        <v>552.76</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="14" t="inlineStr">
-        <is>
-          <t>524 INSURANCE home share (Unit 1 50%, yellow proxy)</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="n">
-        <v>552.7</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>State Farm auto share (personal, excluded)</t>
-        </is>
-      </c>
-      <c r="B41" s="11" t="n">
-        <v>1019.33</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>Geico auto credit (personal, excluded)</t>
-        </is>
-      </c>
-      <c r="B42" s="11" t="n">
-        <v>-540.89</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
+          <t>March HD 100% 524 repairs</t>
+        </is>
+      </c>
+      <c r="B43" s="9" t="n">
+        <v>1358.65</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t>Remaining HD/Lowe’s/IKEA (split pool)</t>
+        </is>
+      </c>
+      <c r="B44" s="9" t="n">
+        <v>1812.46</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
+          <t>524 repairs from remaining 1/3 (then 50/50 U1/U2)</t>
+        </is>
+      </c>
+      <c r="B45" s="9" t="n">
+        <v>604.1799999999999</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="inlineStr">
+        <is>
+          <t>Unit 2 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
+        </is>
+      </c>
+      <c r="B46" s="9" t="n">
+        <v>981.4400000000001</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t>Unit 1 EXTERIOR add (March 50% + remaining 524-share 50%)</t>
+        </is>
+      </c>
+      <c r="B47" s="9" t="n">
+        <v>981.39</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>Personal 1/3 (excluded from P&amp;L)</t>
+        </is>
+      </c>
+      <c r="B48" s="11" t="n">
+        <v>604.16</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>827 N Grove the house 1/3 HD/Lowe’s/IKEA (not Grove Collaborative; not locked $53,660)</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="n">
+        <v>604.12</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>524 Unit 2 SUPPLIES (Grove Collaborative)</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="n">
+        <v>791.21</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>Unit 2 ELECTRIC ComEd Jacob (YELLOW — ask Megan)</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="n">
+        <v>829.15</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>Unit 1 ELECTRIC ComEd Megan (YELLOW — ask Megan)</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="n">
+        <v>1565.26</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>524 INSURANCE home share (Unit 2 50%, yellow proxy)</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="n">
+        <v>552.76</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>524 INSURANCE home share (Unit 1 50%, yellow proxy)</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="n">
+        <v>552.7</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>State Farm auto share (personal, excluded)</t>
+        </is>
+      </c>
+      <c r="B55" s="11" t="n">
+        <v>1019.33</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="10" t="inlineStr">
+        <is>
+          <t>Geico auto credit (personal, excluded)</t>
+        </is>
+      </c>
+      <c r="B56" s="11" t="n">
+        <v>-540.89</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
           <t>Inventory parked (Frame Up + LAMA + Hindman)</t>
         </is>
       </c>
-      <c r="B43" s="9" t="n">
+      <c r="B57" s="9" t="n">
         <v>8043.22</v>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="14" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>Extra Space HOLD</t>
         </is>
       </c>
-      <c r="B44" s="15" t="n">
+      <c r="B58" s="15" t="n">
         <v>360</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="14" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="14" t="inlineStr">
         <is>
           <t>Soldier Field parking HOLD</t>
         </is>
       </c>
-      <c r="B45" s="15" t="n">
+      <c r="B59" s="15" t="n">
         <v>57</v>
+      </c>
+    </row>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Checking inflows 2026-09-18</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="inlineStr">
+        <is>
+          <t>216 Oak Park STR / RENTAL INCOME (cash, incl. Ava yellow)</t>
+        </is>
+      </c>
+      <c r="B62" s="15" t="n">
+        <v>19500</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Delach 8 × $1,450</t>
+        </is>
+      </c>
+      <c r="B63" s="9" t="n">
+        <v>11600</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Ava Hernandez 8 × $500 (ASK roommate)</t>
+        </is>
+      </c>
+      <c r="B64" s="15" t="n">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Joan Friedberger 2 × $1,950 (ASK Dec vs Jan prepaid)</t>
+        </is>
+      </c>
+      <c r="B65" s="15" t="n">
+        <v>3900</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>EPGC Consultant = GCM BOM = 1099-NEC</t>
+        </is>
+      </c>
+      <c r="B66" s="9" t="n">
+        <v>21500</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>GCM reimbursements EXCLUDED (9922 + 8507)</t>
+        </is>
+      </c>
+      <c r="B67" s="11" t="n">
+        <v>5214.69</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="10" t="inlineStr">
+        <is>
+          <t>Bear Creek gift EXCLUDED (4 × $9,500)</t>
+        </is>
+      </c>
+      <c r="B68" s="11" t="n">
+        <v>38000</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="10" t="inlineStr">
+        <is>
+          <t>UTMA Thomas wires EXCLUDED (2 × $5,000)</t>
+        </is>
+      </c>
+      <c r="B69" s="11" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="inlineStr">
+        <is>
+          <t>Freeman’s CIBC $11,000 12/24 HOLD</t>
+        </is>
+      </c>
+      <c r="B70" s="15" t="n">
+        <v>11000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>